<commit_message>
Tag 4: Pivot-Auswertungen zur Inventarnutzung
- Export um person_name ergänzt (auch in den Power-Query-Abfragen)
- Anleitung für vier Pivots inkl. Definition "aktiv" und erwarteter
  Ergebnisse, eigene Fragestellung: Ø Ausleihdauer je Gerätetyp

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/assignments.xlsx
+++ b/docs/exports/assignments.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Ausleihen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ausleihen'!$A$1:$R$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ausleihen'!$A$1:$S$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -449,10 +449,11 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="25" customWidth="1" min="17" max="17"/>
-    <col width="35" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,20 +529,25 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>person_name</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>department</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>person_location</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>damage_note</t>
         </is>
@@ -610,16 +616,21 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Koch, Anna</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Gebäude E</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -686,20 +697,25 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>Koch, Anna</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Gebäude E</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Rückgabe wegen Neugerät</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -764,20 +780,25 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>König, Ben</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Verwaltung</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Gebäude F</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Homeoffice</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -842,16 +863,21 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>Wagner, Eva</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Gebäude E</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -918,20 +944,21 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>Meier, Clara</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>Logistik</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Gebäude H</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Gehäuse am Scanfenster gesprungen</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -996,23 +1023,28 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
+          <t>Schulz, David</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>Logistik</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Gebäude H</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Schichtbetrieb</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R7"/>
+  <autoFilter ref="A1:S7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>